<commit_message>
chore: increasing default core count
</commit_message>
<xml_diff>
--- a/data/output/bfretro.xlsx
+++ b/data/output/bfretro.xlsx
@@ -36,72 +36,72 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Palossand A+SB/ST 1/12/13</t>
+          <t>Blastoise RO+SkB/HC 1/12/15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ghost/ground</t>
+          <t>water/none</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Greedent MS+BS/TBl 4/14/14</t>
+          <t>Kingdra DB+Sw/O 1/13/15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>normal/none</t>
+          <t>water/dragon</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crustle FC+XS/RW 0/14/15</t>
+          <t>Kommo-o DT+UH/ClS 3/15/13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bug/rock</t>
+          <t>dragon/fighting</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cetitan PS+ISp/SP 1/14/11</t>
+          <t>Grumpig Psy+SB/DyP 6/14/13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ice/none</t>
+          <t>psychic/none</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Annihilape LK+RF/CC 3/11/15</t>
+          <t>Skeledirge I+TSo/SB 0/15/15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>fighting/ghost</t>
+          <t>fire/ghost</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Roserade PSt+WBF/LfS 0/14/12</t>
+          <t>Golisopod FC+XS/AJ 1/14/15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>grass/poison</t>
+          <t>bug/water</t>
         </is>
       </c>
     </row>
@@ -131,7 +131,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>377.4611398963731</v>
+        <v>227.57894736842104</v>
       </c>
     </row>
     <row r="3">
@@ -141,7 +141,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>179.29403210772855</v>
+        <v>197.9092756412052</v>
       </c>
     </row>
     <row r="4">
@@ -151,7 +151,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>88.48659003831418</v>
+        <v>181.0</v>
       </c>
     </row>
     <row r="5">
@@ -161,7 +161,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>192.2466590025347</v>
+        <v>200.04721638481848</v>
       </c>
     </row>
     <row r="6">
@@ -171,7 +171,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>807.2518518518518</v>
+        <v>819.2777777777777</v>
       </c>
     </row>
     <row r="7">
@@ -181,7 +181,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>118</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -191,7 +191,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>0.8740740740740741</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="9">
@@ -201,7 +201,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>45</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -211,7 +211,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>741.6962962962963</v>
+        <v>752.6111111111111</v>
       </c>
     </row>
     <row r="11">
@@ -261,7 +261,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>135</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -271,7 +271,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>135</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -281,7 +281,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>100</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18">
@@ -321,7 +321,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>96.3</v>
+        <v>88.6</v>
       </c>
     </row>
     <row r="22">
@@ -331,7 +331,7 @@
         </is>
       </c>
       <c r="B22">
-        <v>69.376</v>
+        <v>80.25454545454545</v>
       </c>
     </row>
     <row r="23">
@@ -341,7 +341,7 @@
         </is>
       </c>
       <c r="B23">
-        <v>26.7</v>
+        <v>66.9</v>
       </c>
     </row>
     <row r="24">
@@ -363,7 +363,7 @@
         </is>
       </c>
       <c r="B25">
-        <v>79.35000000000001</v>
+        <v>77.88333333333334</v>
       </c>
     </row>
     <row r="26">
@@ -373,7 +373,7 @@
         </is>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -383,7 +383,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>0.0</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="28">
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="B28">
-        <v>135</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29">
@@ -403,7 +403,7 @@
         </is>
       </c>
       <c r="B29">
-        <v>686.7045454545453</v>
+        <v>715.1666666666666</v>
       </c>
     </row>
   </sheetData>
@@ -445,7 +445,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -462,7 +462,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -479,7 +479,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -516,7 +516,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Palossand A+SB/ST 1/12/13, Cetitan PS+ISp/SP 1/14/11, Roserade PSt+WBF/LfS 0/14/12</t>
+          <t>Blastoise RO+SkB/HC 1/12/15, Kommo-o DT+UH/ClS 3/15/13, Grumpig Psy+SB/DyP 6/14/13</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Palossand A+SB/ST 1/12/13, Greedent MS+BS/TBl 4/14/14, Annihilape LK+RF/CC 3/11/15</t>
+          <t>Kommo-o DT+UH/ClS 3/15/13, Grumpig Psy+SB/DyP 6/14/13, Skeledirge I+TSo/SB 0/15/15</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Greedent MS+BS/TBl 4/14/14, Cetitan PS+ISp/SP 1/14/11, Annihilape LK+RF/CC 3/11/15</t>
+          <t>Blastoise RO+SkB/HC 1/12/15, Kingdra DB+Sw/O 1/13/15, Grumpig Psy+SB/DyP 6/14/13</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Crustle FC+XS/RW 0/14/15, Cetitan PS+ISp/SP 1/14/11, Annihilape LK+RF/CC 3/11/15</t>
+          <t>Blastoise RO+SkB/HC 1/12/15, Grumpig Psy+SB/DyP 6/14/13, Golisopod FC+XS/AJ 1/14/15</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,57 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Greedent MS+BS/TBl 4/14/14, Crustle FC+XS/RW 0/14/15, Annihilape LK+RF/CC 3/11/15</t>
+          <t>Grumpig Psy+SB/DyP 6/14/13, Skeledirge I+TSo/SB 0/15/15, Golisopod FC+XS/AJ 1/14/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Blastoise RO+SkB/HC 1/12/15, Kingdra DB+Sw/O 1/13/15, Kommo-o DT+UH/ClS 3/15/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kingdra DB+Sw/O 1/13/15, Kommo-o DT+UH/ClS 3/15/13, Grumpig Psy+SB/DyP 6/14/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kingdra DB+Sw/O 1/13/15, Kommo-o DT+UH/ClS 3/15/13, Skeledirge I+TSo/SB 0/15/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kommo-o DT+UH/ClS 3/15/13, Grumpig Psy+SB/DyP 6/14/13, Golisopod FC+XS/AJ 1/14/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Blastoise RO+SkB/HC 1/12/15, Kingdra DB+Sw/O 1/13/15, Golisopod FC+XS/AJ 1/14/15</t>
         </is>
       </c>
     </row>
@@ -592,180 +642,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kingdra DB+Sw/O 0/15/15</t>
+          <t>Kommo-o DT+ClS/UH 4/12/13</t>
         </is>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Drifblim A+IW/SB 1/15/15</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Tentacruel Ac+Sc/Pbk 0/13/15</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Kommo-o DT+ClS/UH 0/11/14</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Gyarados (Shadow) DB+AT/Tw 0/15/14</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Golisopod FC+XS/AJ 1/14/15</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Giratina (Origin) SC+SB/DgP 1/12/13</t>
-        </is>
-      </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Giratina (Origin) SC+SB/DgP 1/12/13</t>
-        </is>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Poliwrath MS+IW/DyP 0/14/14</t>
-        </is>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Walrein PS+ISp/Eq 0/15/15</t>
-        </is>
-      </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>0-shield only Grumpig Psy+SB/DyP 6/14/13 | 1-shield only Grumpig Psy+SB/DyP 6/14/13</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
chore: increasing default core count (#3)
</commit_message>
<xml_diff>
--- a/data/output/bfretro.xlsx
+++ b/data/output/bfretro.xlsx
@@ -36,72 +36,72 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Palossand A+SB/ST 1/12/13</t>
+          <t>Blastoise RO+SkB/HC 1/12/15</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>ghost/ground</t>
+          <t>water/none</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Greedent MS+BS/TBl 4/14/14</t>
+          <t>Kingdra DB+Sw/O 1/13/15</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>normal/none</t>
+          <t>water/dragon</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Crustle FC+XS/RW 0/14/15</t>
+          <t>Kommo-o DT+UH/ClS 3/15/13</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>bug/rock</t>
+          <t>dragon/fighting</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Cetitan PS+ISp/SP 1/14/11</t>
+          <t>Grumpig Psy+SB/DyP 6/14/13</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>ice/none</t>
+          <t>psychic/none</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Annihilape LK+RF/CC 3/11/15</t>
+          <t>Skeledirge I+TSo/SB 0/15/15</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>fighting/ghost</t>
+          <t>fire/ghost</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Roserade PSt+WBF/LfS 0/14/12</t>
+          <t>Golisopod FC+XS/AJ 1/14/15</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>grass/poison</t>
+          <t>bug/water</t>
         </is>
       </c>
     </row>
@@ -131,7 +131,7 @@
         </is>
       </c>
       <c r="B2">
-        <v>377.4611398963731</v>
+        <v>227.57894736842104</v>
       </c>
     </row>
     <row r="3">
@@ -141,7 +141,7 @@
         </is>
       </c>
       <c r="B3">
-        <v>179.29403210772855</v>
+        <v>197.9092756412052</v>
       </c>
     </row>
     <row r="4">
@@ -151,7 +151,7 @@
         </is>
       </c>
       <c r="B4">
-        <v>88.48659003831418</v>
+        <v>181.0</v>
       </c>
     </row>
     <row r="5">
@@ -161,7 +161,7 @@
         </is>
       </c>
       <c r="B5">
-        <v>192.2466590025347</v>
+        <v>200.04721638481848</v>
       </c>
     </row>
     <row r="6">
@@ -171,7 +171,7 @@
         </is>
       </c>
       <c r="B6">
-        <v>807.2518518518518</v>
+        <v>819.2777777777777</v>
       </c>
     </row>
     <row r="7">
@@ -181,7 +181,7 @@
         </is>
       </c>
       <c r="B7">
-        <v>118</v>
+        <v>16</v>
       </c>
     </row>
     <row r="8">
@@ -191,7 +191,7 @@
         </is>
       </c>
       <c r="B8">
-        <v>0.8740740740740741</v>
+        <v>0.8888888888888888</v>
       </c>
     </row>
     <row r="9">
@@ -201,7 +201,7 @@
         </is>
       </c>
       <c r="B9">
-        <v>45</v>
+        <v>6</v>
       </c>
     </row>
     <row r="10">
@@ -211,7 +211,7 @@
         </is>
       </c>
       <c r="B10">
-        <v>741.6962962962963</v>
+        <v>752.6111111111111</v>
       </c>
     </row>
     <row r="11">
@@ -261,7 +261,7 @@
         </is>
       </c>
       <c r="B15">
-        <v>135</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -271,7 +271,7 @@
         </is>
       </c>
       <c r="B16">
-        <v>135</v>
+        <v>16</v>
       </c>
     </row>
     <row r="17">
@@ -281,7 +281,7 @@
         </is>
       </c>
       <c r="B17">
-        <v>100</v>
+        <v>11</v>
       </c>
     </row>
     <row r="18">
@@ -321,7 +321,7 @@
         </is>
       </c>
       <c r="B21">
-        <v>96.3</v>
+        <v>88.6</v>
       </c>
     </row>
     <row r="22">
@@ -331,7 +331,7 @@
         </is>
       </c>
       <c r="B22">
-        <v>69.376</v>
+        <v>80.25454545454545</v>
       </c>
     </row>
     <row r="23">
@@ -341,7 +341,7 @@
         </is>
       </c>
       <c r="B23">
-        <v>26.7</v>
+        <v>66.9</v>
       </c>
     </row>
     <row r="24">
@@ -363,7 +363,7 @@
         </is>
       </c>
       <c r="B25">
-        <v>79.35000000000001</v>
+        <v>77.88333333333334</v>
       </c>
     </row>
     <row r="26">
@@ -373,7 +373,7 @@
         </is>
       </c>
       <c r="B26">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="27">
@@ -383,7 +383,7 @@
         </is>
       </c>
       <c r="B27">
-        <v>0.0</v>
+        <v>0.1111111111111111</v>
       </c>
     </row>
     <row r="28">
@@ -393,7 +393,7 @@
         </is>
       </c>
       <c r="B28">
-        <v>135</v>
+        <v>18</v>
       </c>
     </row>
     <row r="29">
@@ -403,7 +403,7 @@
         </is>
       </c>
       <c r="B29">
-        <v>686.7045454545453</v>
+        <v>715.1666666666666</v>
       </c>
     </row>
   </sheetData>
@@ -445,7 +445,7 @@
         <v>0</v>
       </c>
       <c r="B2">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C2">
         <v>0</v>
@@ -462,7 +462,7 @@
         <v>1</v>
       </c>
       <c r="B3">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C3">
         <v>0</v>
@@ -479,7 +479,7 @@
         <v>2</v>
       </c>
       <c r="B4">
-        <v>45</v>
+        <v>6</v>
       </c>
       <c r="C4">
         <v>0</v>
@@ -516,7 +516,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Palossand A+SB/ST 1/12/13, Cetitan PS+ISp/SP 1/14/11, Roserade PSt+WBF/LfS 0/14/12</t>
+          <t>Blastoise RO+SkB/HC 1/12/15, Kommo-o DT+UH/ClS 3/15/13, Grumpig Psy+SB/DyP 6/14/13</t>
         </is>
       </c>
     </row>
@@ -526,7 +526,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Palossand A+SB/ST 1/12/13, Greedent MS+BS/TBl 4/14/14, Annihilape LK+RF/CC 3/11/15</t>
+          <t>Kommo-o DT+UH/ClS 3/15/13, Grumpig Psy+SB/DyP 6/14/13, Skeledirge I+TSo/SB 0/15/15</t>
         </is>
       </c>
     </row>
@@ -536,7 +536,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Greedent MS+BS/TBl 4/14/14, Cetitan PS+ISp/SP 1/14/11, Annihilape LK+RF/CC 3/11/15</t>
+          <t>Blastoise RO+SkB/HC 1/12/15, Kingdra DB+Sw/O 1/13/15, Grumpig Psy+SB/DyP 6/14/13</t>
         </is>
       </c>
     </row>
@@ -546,7 +546,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Crustle FC+XS/RW 0/14/15, Cetitan PS+ISp/SP 1/14/11, Annihilape LK+RF/CC 3/11/15</t>
+          <t>Blastoise RO+SkB/HC 1/12/15, Grumpig Psy+SB/DyP 6/14/13, Golisopod FC+XS/AJ 1/14/15</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,57 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Greedent MS+BS/TBl 4/14/14, Crustle FC+XS/RW 0/14/15, Annihilape LK+RF/CC 3/11/15</t>
+          <t>Grumpig Psy+SB/DyP 6/14/13, Skeledirge I+TSo/SB 0/15/15, Golisopod FC+XS/AJ 1/14/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Blastoise RO+SkB/HC 1/12/15, Kingdra DB+Sw/O 1/13/15, Kommo-o DT+UH/ClS 3/15/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Kingdra DB+Sw/O 1/13/15, Kommo-o DT+UH/ClS 3/15/13, Grumpig Psy+SB/DyP 6/14/13</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Kingdra DB+Sw/O 1/13/15, Kommo-o DT+UH/ClS 3/15/13, Skeledirge I+TSo/SB 0/15/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Kommo-o DT+UH/ClS 3/15/13, Grumpig Psy+SB/DyP 6/14/13, Golisopod FC+XS/AJ 1/14/15</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Blastoise RO+SkB/HC 1/12/15, Kingdra DB+Sw/O 1/13/15, Golisopod FC+XS/AJ 1/14/15</t>
         </is>
       </c>
     </row>
@@ -592,180 +642,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Kingdra DB+Sw/O 0/15/15</t>
+          <t>Kommo-o DT+ClS/UH 4/12/13</t>
         </is>
       </c>
       <c r="B2">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Drifblim A+IW/SB 1/15/15</t>
-        </is>
-      </c>
-      <c r="B3">
-        <v>0</v>
-      </c>
-      <c r="C3">
-        <v>0</v>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Tentacruel Ac+Sc/Pbk 0/13/15</t>
-        </is>
-      </c>
-      <c r="B4">
-        <v>0</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Kommo-o DT+ClS/UH 0/11/14</t>
-        </is>
-      </c>
-      <c r="B5">
-        <v>0</v>
-      </c>
-      <c r="C5">
-        <v>0</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Gyarados (Shadow) DB+AT/Tw 0/15/14</t>
-        </is>
-      </c>
-      <c r="B6">
-        <v>0</v>
-      </c>
-      <c r="C6">
-        <v>0</v>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Golisopod FC+XS/AJ 1/14/15</t>
-        </is>
-      </c>
-      <c r="B7">
-        <v>0</v>
-      </c>
-      <c r="C7">
-        <v>0</v>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Giratina (Origin) SC+SB/DgP 1/12/13</t>
-        </is>
-      </c>
-      <c r="B8">
-        <v>0</v>
-      </c>
-      <c r="C8">
-        <v>0</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Giratina (Origin) SC+SB/DgP 1/12/13</t>
-        </is>
-      </c>
-      <c r="B9">
-        <v>0</v>
-      </c>
-      <c r="C9">
-        <v>0</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>Poliwrath MS+IW/DyP 0/14/14</t>
-        </is>
-      </c>
-      <c r="B10">
-        <v>0</v>
-      </c>
-      <c r="C10">
-        <v>0</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>n/a</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>Walrein PS+ISp/Eq 0/15/15</t>
-        </is>
-      </c>
-      <c r="B11">
-        <v>0</v>
-      </c>
-      <c r="C11">
-        <v>0</v>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>n/a</t>
+          <t>0-shield only Grumpig Psy+SB/DyP 6/14/13 | 1-shield only Grumpig Psy+SB/DyP 6/14/13</t>
         </is>
       </c>
     </row>

</xml_diff>